<commit_message>
Close P0 Phase 0–1 locally and declare Langfuse metadata-only.
Publish the dispute demo contract, BigQuery problem baseline, and a disabled Langfuse exporter so delivery can advance without shipping secrets or content telemetry.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tareas - Revisado" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa Factored" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tareas - Revisado" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mapa Factored" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -666,10 +666,14 @@
       </c>
       <c r="H2" s="26" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I2" s="18" t="n"/>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I2" s="18" t="inlineStr">
+        <is>
+          <t>Consulta versionada p0-01-contact-motive-distribution sobre factored-hackathon.hackathon; distribución de motivos Transactions publicada en docs/phase1-problem-baseline-20261004.md (agregados, sin PII).</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="86.25" customHeight="1" s="19">
       <c r="A3" s="26" t="inlineStr">
@@ -709,10 +713,14 @@
       </c>
       <c r="H3" s="26" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I3" s="18" t="n"/>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I3" s="18" t="inlineStr">
+        <is>
+          <t>Consultas p0-02-population-denominator y p0-02-volume-severity-temporality; volumen/severidad/temporalidad y denominadores en el mismo snapshot (TZ America/Lima).</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="60" customHeight="1" s="19">
       <c r="A4" s="26" t="inlineStr">
@@ -752,12 +760,12 @@
       </c>
       <c r="H4" s="26" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I4" s="26" t="inlineStr">
         <is>
-          <t>Cliente: Banco Usuario: Banco y Cliente de banco. Métrica a mejorar: Tiempo de resolucion de incidente</t>
+          <t>Product brief publicado en docs/product/dispute-transaction-support-brief.md: Banco, cliente/operador, KPI tiempo de resolución, trade-offs; baseline cuantitativo remite a P0-05.</t>
         </is>
       </c>
     </row>
@@ -799,12 +807,12 @@
       </c>
       <c r="H5" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I5" s="26" t="inlineStr">
         <is>
-          <t>Aplicación de dos usuarios: cliente y backoffice. Alcance: Autenticación (emular) No alcance:</t>
+          <t>Matriz v1 Zod en capability-matrix.ts + mirror docs/product/dispute-capability-matrix-v1.md; cada acción con roles, capability, allowedData, requiredEvidence y mock effect=none; aliases customer/backoffice.</t>
         </is>
       </c>
     </row>
@@ -846,12 +854,12 @@
       </c>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I6" s="26" t="inlineStr">
         <is>
-          <t>Investigar el promedio de resolución general</t>
+          <t>Baseline manual resolution_days: terminales Resolved/Closed, n=3165, mean≈15.4, p50=15, p90=27, sla_breach≈0.19; query_id p0-05-manual-resolution-baseline.</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2076,14 @@
       </c>
       <c r="H32" s="26" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I32" s="18" t="n"/>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I32" s="18" t="inlineStr">
+        <is>
+          <t>Pack sintético versionado dispute-demo-v1 (actores, sesiones, txn/dispute/case/evidencia) en domain/demo-fixtures.ts; createDemoRuntime lo consume; sin PII bancaria real.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="72.75" customHeight="1" s="19">
       <c r="A33" s="26" t="inlineStr">

</xml_diff>

<commit_message>
docs: reconcile P0 task status with GCP inventory
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tareas - Revisado" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mapa Factored" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tareas - Revisado" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa Factored" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -2166,10 +2166,14 @@
       </c>
       <c r="H34" s="26" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I34" s="18" t="n"/>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="I34" s="18" t="inlineStr">
+        <is>
+          <t>OTel/Langfuse Cloud US metadata-only, evaluadores baseline y persistencia BigQuery saneada implementados; Terraform declara dataset/tabla y preflight valida. Falta configurar secretos/flags autorizados, aplicar infraestructura y validar emisión en staging.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="94.5" customHeight="1" s="19">
       <c r="A35" s="26" t="inlineStr">
@@ -2299,12 +2303,12 @@
       </c>
       <c r="H37" s="26" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="I37" s="26" t="inlineStr">
         <is>
-          <t>ADR 0014 / ADR 0017 / ADR 0020</t>
+          <t>Terraform declara referencias Secret Manager versionables, IAM mínimo para backend (Firestore, BigQuery, Vertex y writer de evaluaciones) y VPC/Valkey; falta crear o importar recursos reales, revisar plan autorizado y aplicar.</t>
         </is>
       </c>
     </row>
@@ -2346,12 +2350,12 @@
       </c>
       <c r="H38" s="26" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="I38" s="26" t="inlineStr">
         <is>
-          <t>ADR 0014 / ADR 0017 / ADR 0020</t>
+          <t>Dockerfiles, Artifact Registry, Cloud Run/Job Terraform y preflight productivo están validados sin apply; faltan digests reales, terraform plan/apply autorizado, publicación de grafo GCS y smoke Cloud Run.</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3423,7 @@
       </c>
       <c r="I62" s="26" t="inlineStr">
         <is>
-          <t>Ledger e idempotencia del contrato local están cubiertos; falta worker administrado ADR 0020 con Eventarc/Cloud Tasks y BigQuery.</t>
+          <t>Ledger e idempotencia del contrato local están cubiertos; falta worker administrado ADR 0020 con Storage Transfer Service, Eventarc, Cloud Tasks, copia verified/ y carga BigQuery.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: refresh GCP inventory after Publish images recovery
Record baseline chat + KG live state, CI runner note, and keep cloud P0 rows IN PROGRESS.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -1329,7 +1329,7 @@
       </c>
       <c r="I16" s="18" t="inlineStr">
         <is>
-          <t>Catálogo KG cerrado y versionado implementado localmente; falta publicación GCS y lease Firestore.</t>
+          <t>Catálogo KG cerrado y versionado; artefacto GCS demo-bankai/current.json (graph-20261004-fullpop-ci) publicado. DoD abierto: lease Firestore y habilitación productiva del catálogo.</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="I29" s="18" t="inlineStr">
         <is>
-          <t>KG-RAG local, catálogo, validación de artefacto y operaciones allowlisted implementados; publicación GCS/lease Firestore pendientes.</t>
+          <t>KG-RAG local/allowlist implementados; artefacto GCS publicado. DoD abierto: lease Firestore, KG-RAG productivo cerrado y smoke autorizado (KG_RAG_LOCAL_ENABLED=false en Cloud Run).</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="I38" s="26" t="inlineStr">
         <is>
-          <t>Dockerfiles, Artifact Registry, Cloud Run/Job Terraform y preflight productivo están validados sin apply; faltan digests reales, terraform plan/apply autorizado, publicación de grafo GCS y smoke Cloud Run.</t>
+          <t>Cloud Run bankai-backend Ready (rev bankai-backend-00010-zxt, imagen sha256:76211ea7…0044) con chat baseline; Publish images 37366452866 success tras reintento por runner. Job bankai-pipeline creado sin ejecuciones observadas. DoD abierto: terraform plan/apply reconciliado (correlador→Secret Manager) y cadena de ingesta.</t>
         </is>
       </c>
     </row>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="I59" s="26" t="inlineStr">
         <is>
-          <t>Compilación local del grafo y publicación de artefacto emulado implementadas; falta publicación productiva GCS.</t>
+          <t>Compilación local + publicación GCS de graph-20261004-fullpop-ci (msgpack/manifest/catalog/current.json). DoD abierto: KDD sobre capas curadas y lease Firestore.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: materialize curated stg/aux/cur from canonical BigQuery
Enable authorized --canonical-prepare to close Fase 2 (P0-06–10, P0-44) without waiting on ADR 0020 raw ingest.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tareas - Revisado" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa Factored" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tareas - Revisado" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mapa Factored" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -901,12 +901,12 @@
       </c>
       <c r="H7" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I7" s="18" t="inlineStr">
         <is>
-          <t>Contrato local por tabla y validación de esquema implementados; faltan metadata, freshness y drift sobre BigQuery autorizado.</t>
+          <t>Contratos dispute-transaction-v1 validados contra INFORMATION_SCHEMA de factored-hackathon.hackathon (TX/complaints/CCI/surveys) en prepare-20261005-canonical; drift falla cerrado.</t>
         </is>
       </c>
     </row>
@@ -948,12 +948,12 @@
       </c>
       <c r="H8" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I8" s="18" t="inlineStr">
         <is>
-          <t>Perfilado y validaciones locales cubiertos por pruebas; falta ejecutar sobre metadata y snapshots BigQuery autorizados.</t>
+          <t>Perfiles agregados BQ (row_count, null_counts, duplicate PK, freshness min/max) en prepare-manifest; sin valores de fila ni IDs.</t>
         </is>
       </c>
     </row>
@@ -995,12 +995,12 @@
       </c>
       <c r="H9" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I9" s="18" t="inlineStr">
         <is>
-          <t>Pendiente de vistas curadas versionadas en BigQuery; los contratos cerrados ya documentan las columnas esperadas.</t>
+          <t>Datasets stg/aux/cur materializados con proyección mínima de contratos; stg dedupe por PK+freshness; sin columnas de texto libre.</t>
         </is>
       </c>
     </row>
@@ -1042,12 +1042,12 @@
       </c>
       <c r="H10" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I10" s="18" t="inlineStr">
         <is>
-          <t>Preparación determinista local implementada: deduplicación, normalización, imputación y rechazo de claves/freshness inválidos.</t>
+          <t>Pipeline canónico autorizado hackathon→stg→aux→cur vía bankai-pipeline --canonical-prepare run_id=prepare-20261005-canonical; conteos TX=4,425,008 complaints=67,095.</t>
         </is>
       </c>
     </row>
@@ -1089,12 +1089,12 @@
       </c>
       <c r="H11" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I11" s="26" t="inlineStr">
         <is>
-          <t>Lineage y manifest saneado implementados con hash, generación, watermark, transforms y content hash; falta conectarlo al worker ADR 0020.</t>
+          <t>Lineage bankai-lineage-v1 + cur.preparation_runs (metadata-only) y artifacts/prepare/&lt;run-id&gt;/prepare-manifest.json; contains_source_values=false.</t>
         </is>
       </c>
     </row>
@@ -2667,12 +2667,12 @@
       </c>
       <c r="H45" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I45" s="18" t="inlineStr">
         <is>
-          <t>Reglas de imputación reproducibles implementadas en preparación local; falta ejecución sobre tablas staging/curadas BigQuery.</t>
+          <t>Imputación reproducible en cur.* con *_was_imputed (mediana/moda por grupo + UNKNOWN); p.ej. cur.complaints claimed_amount_was_imputed=45,344.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: run KDD and publish curated KG from BigQuery cur
Point offline configs at cur, fix category case filters and KDD JSON datetime serialization, and close Fase 4 with leased GCS publication.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -1136,12 +1136,12 @@
       </c>
       <c r="H12" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I12" s="26" t="inlineStr">
         <is>
-          <t>CRISP-DM/KDD documentado en el modelo operativo y enlazado desde la guía del pipeline.</t>
+          <t>CRISP-DM/KDD documentado; fuente post-Fase-2 = dataset cur (configs *.toml.example).</t>
         </is>
       </c>
     </row>
@@ -1183,12 +1183,12 @@
       </c>
       <c r="H13" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I13" s="26" t="inlineStr">
         <is>
-          <t>KDD reproducible y comparación Apriori/FP-Growth implementados localmente; ejecución sobre datos curados cloud sigue pendiente.</t>
+          <t>KDD kdd-20261005-cur sobre factored-hackathon.cur (TX 4.4M + complaints TRANSACTIONS 13.5k); filtros categoría case-insensitive.</t>
         </is>
       </c>
     </row>
@@ -1230,12 +1230,12 @@
       </c>
       <c r="H14" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I14" s="18" t="inlineStr">
         <is>
-          <t>Ontología agregada del grafo implementada para población, feature, valor, target, regla, caso y corrida de modelo.</t>
+          <t>Ontología agregada usada por compile-graph graph-20261005-cur (Population/Feature/Rule/…).</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="H15" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I15" s="26" t="inlineStr">
         <is>
-          <t>Compilador local implementado; publica artefactos versionados y conserva sólo reglas corroboradas por Apriori y FP-Growth.</t>
+          <t>Compilador produjo graph-v1.msgpack + graph-manifest.json en artifacts/graph/graph-20261005-cur con consenso Apriori∩FP-Growth∩Eclat.</t>
         </is>
       </c>
     </row>
@@ -1324,12 +1324,12 @@
       </c>
       <c r="H16" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I16" s="18" t="inlineStr">
         <is>
-          <t>Catálogo KG cerrado y versionado; artefacto GCS demo-bankai/current.json (graph-20261004-fullpop-ci) publicado. DoD abierto: lease Firestore y habilitación productiva del catálogo.</t>
+          <t>Catálogo kg-operation-catalog publicado en GCS demo-bankai/graph-20261005-cur; current.json actualizado con lease Firestore.</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1935,12 @@
       </c>
       <c r="H29" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I29" s="18" t="inlineStr">
         <is>
-          <t>KG-RAG local/allowlist implementados; artefacto GCS publicado. DoD abierto: lease Firestore, KG-RAG productivo cerrado y smoke autorizado (KG_RAG_LOCAL_ENABLED=false en Cloud Run).</t>
+          <t>Consumer Cloud Run GCS_ENABLED + GCS_GRAPH_BUCKET/demo-bankai; KG_RAG_LOCAL_ENABLED=false; health 200 tras current.json graph-20261005-cur.</t>
         </is>
       </c>
     </row>
@@ -3230,12 +3230,12 @@
       </c>
       <c r="H58" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I58" s="26" t="inlineStr">
         <is>
-          <t>Etapas KDD y baselines C1–C5 están disponibles como comandos offline; falta correr el conjunto cloud autorizado.</t>
+          <t>C1–C5 ejecutados sobre cur (cN-20261005-cur) + evaluate-supervised-suite suite-20261005-cur.</t>
         </is>
       </c>
     </row>
@@ -3277,12 +3277,12 @@
       </c>
       <c r="H59" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I59" s="26" t="inlineStr">
         <is>
-          <t>Compilación local + publicación GCS de graph-20261004-fullpop-ci (msgpack/manifest/catalog/current.json). DoD abierto: KDD sobre capas curadas y lease Firestore.</t>
+          <t>Grafo compilado desde kdd-20261005-cur + suite; publish GCS con lease (run graph-20261005-cur). graph-diff vs fullpop informativo: gate holdout_stable falló (esperado cur vs hackathon).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: seed Firestore demo identity and productive store evidence
Wire demo/baseline RBAC overlays and SessionManager tests without enabling agentic chat, and add CI dry-run plus authorized execute workflow.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -1606,12 +1606,12 @@
       </c>
       <c r="H22" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I22" s="18" t="inlineStr">
         <is>
-          <t>API Bun/Fastify, OpenAPI y contratos de chat disponibles; faltan validaciones de integración productiva.</t>
+          <t>OpenAPI + demo/session smoke (inject + docs Cloud Run); DEMO_AUTH+baseline intactos en staging.</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="I23" s="18" t="inlineStr">
         <is>
-          <t>Auth/RBAC y actores demo están cubiertos por contratos; Firebase Auth productivo continúa pendiente.</t>
+          <t>RBAC Firestore seed (user_profiles/bindings); Firebase Auth bloqueado Harumi P0-17.</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="I25" s="18" t="inlineStr">
         <is>
-          <t>Input Rail, sanitización y límites están presentes; falta validar composición productiva completa.</t>
+          <t>Rails/policy en suite integración demo (sin agentic); Model Armor cloud pendiente Alexandra.</t>
         </is>
       </c>
     </row>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="I26" s="18" t="inlineStr">
         <is>
-          <t>Routing JEV jerárquico y selección cerrada implementados; faltan proveedores productivos y pruebas de integración autorizadas.</t>
+          <t>JEV jerárquico en código; sin proveedor productivo nuevo; agentic no activado.</t>
         </is>
       </c>
     </row>
@@ -1846,7 +1846,7 @@
       </c>
       <c r="I27" s="18" t="inlineStr">
         <is>
-          <t>Policy Engine y Tool Gateway tienen contratos y dobles; falta activación/composición productiva.</t>
+          <t>Policy/Tool Gateway evidenciado en tests demo; composición agentic no cerrada.</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="I30" s="18" t="inlineStr">
         <is>
-          <t>Output Rail y generación saneada están implementados; faltan pruebas productivas contra proveedores autorizados.</t>
+          <t>Output rail en suite demo/baseline; Model Armor cloud no verificado.</t>
         </is>
       </c>
     </row>
@@ -2029,12 +2029,12 @@
       </c>
       <c r="H31" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I31" s="18" t="inlineStr">
         <is>
-          <t>Puertos y dobles para Firestore/Valkey están presentes; integración real y configuración durable siguen pendientes.</t>
+          <t>Firestore conversation_snapshots + Valkey SessionManager wiring; seed perfiles; índice declarado (sin TF apply).</t>
         </is>
       </c>
     </row>
@@ -2256,12 +2256,12 @@
       </c>
       <c r="H36" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I36" s="18" t="inlineStr">
         <is>
-          <t>Pruebas de contrato OpenAPI y suites backend ejecutadas; falta completar integración con servicios productivos.</t>
+          <t>Contract/integration tests ampliados (seed dry-run CI, productive stores demo, OpenAPI).</t>
         </is>
       </c>
     </row>
@@ -3324,12 +3324,12 @@
       </c>
       <c r="H60" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I60" s="18" t="inlineStr">
         <is>
-          <t>SessionManager, contratos y aislamiento de demo están implementados; falta persistencia Firestore y coordinación Valkey reales.</t>
+          <t>SessionManager Valkey + perfiles Firestore; cookie __Host-session Secure; smoke documentado.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: gate P0 eval matrix 48 core + 5 KG C1–C5 in CI
Add eval:gate contract checks so PRs enforce the deterministic informational matrix without blocking on score thresholds or emit.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -3371,12 +3371,12 @@
       </c>
       <c r="H61" s="26" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="I61" s="26" t="inlineStr">
         <is>
-          <t>Matriz informativa implementada con 48 casos core + 5 extensiones KG C1–C5; falta CI y baseline humano.</t>
+          <t>COMPLETED: CI gate eval:run + eval:gate con 48 core + 5 extensiones KG C1–C5 (contrato informational; sin --emit). Baseline humana / umbrales bloqueantes quedan como seguimiento ADR 0015 / P0-39. Matriz=trayectorias sintéticas; NL de producto fuera de alcance P0-48.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add local A/B compare for baseline vs control plane
Run synthetic research prompts through both pipelines offline and persist sanitized JSONL under .local/eval-ab without cloud writes or reopening P0-48.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13.25" customWidth="1" style="18" min="1" max="1"/>
@@ -3486,6 +3486,53 @@
       <c r="F68" s="30" t="n"/>
       <c r="G68" s="29" t="n"/>
       <c r="I68" s="32" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>P0-50</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Comparar baseline vs control plane (A/B local).</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CLI eval:compare con escenarios de prompts sintéticos (phase-1 Structured + phase-2 C1–C5/research). File sink local; sin persist BQ. Completitud técnica; juez semántico skipped.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Bun 1.4 · TypeScript · bun test · AgentControlService · BaselineConversationRunner</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Ricardo</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Done: bun run eval:compare genera runs/metrics/summary saneados en .local/eval-ab; same snapshot A/B; controlled gates vs baseline ungated; sin PII/prompts en artefactos; P0-48 intacto.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Local A/B file sink listo (eval:compare). BQ vista segura/--persist diferido. P0-48 no reabierto.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
feat: drop /v1/items scaffold and expand A/B corpus to 128 ES/PT prompts
Remove the demo items CRUD from OpenAPI and runtime, reconcile P0 status
handoffs, and grow local baseline vs control-plane evaluation to 64 Spanish
and 64 Portuguese scenarios including HITL escalation casuistics.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/factored_tasks.xlsx
+++ b/docs/planning/to-adopt/factored_tasks.xlsx
@@ -1376,7 +1376,7 @@
       </c>
       <c r="I17" s="26" t="inlineStr">
         <is>
-          <t>ADR 0021</t>
+          <t>ADR 0021. Scaffold ausente. Contrato/smoke desbloqueo: docs/handoffs/frontend-auth-smoke-p0-16-22-38.md (2026-10-05).</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="I18" s="26" t="inlineStr">
         <is>
-          <t>ADR 0021</t>
+          <t>ADR 0021. Firebase Auth demo pendiente Harumi. Backend listo para verificar ID token tras P0-17; smoke en handoff frontend-auth.</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="I19" s="26" t="inlineStr">
         <is>
-          <t>ADR 0021</t>
+          <t>ADR 0021. Chat cliente pendiente scaffold. Backend OpenAPI/AsyncAPI + WS demo documentados en app/frontend/README y handoff smoke.</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="I20" s="26" t="inlineStr">
         <is>
-          <t>ADR 0021</t>
+          <t>ADR 0021. Consola operador pendiente. Eventos HITL (hitl.created/backoffice.alert) expuestos por API/WS; UI Harumi.</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="I21" s="26" t="inlineStr">
         <is>
-          <t>ADR 0021</t>
+          <t>ADR 0021. Estados UI transversales pendientes scaffold. Mapa estados control plane en ADR 0004/0007.</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="I23" s="18" t="inlineStr">
         <is>
-          <t>RBAC Firestore seed (user_profiles/bindings); Firebase Auth bloqueado Harumi P0-17.</t>
+          <t>RBAC Firestore seed (user_profiles/bindings) OK. Firebase Auth E2E bloqueado Harumi P0-17. Smoke: docs/handoffs/frontend-auth-smoke-p0-16-22-38.md.</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1705,7 @@
       </c>
       <c r="I24" s="18" t="inlineStr">
         <is>
-          <t>StateGraph explícito con rutas llm/database/relations/ood y orden kg_catalog → kg_jev → policy → kg_rag implementado.</t>
+          <t>IN PROGRESS (no COMPLETED): código en main PR#13 — StateGraph+ControlPlaneConversationRunner+requiresEscalation→escalation.request+casuísticas/HITL. Staging sigue CHAT_PIPELINE=baseline. Cutover: docs/handoffs/agentic-control-plane-cutover.md. Reconciliación: docs/task-status-reconciled-20261005.md.</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="I25" s="18" t="inlineStr">
         <is>
-          <t>Rails/policy en suite integración demo (sin agentic); Model Armor cloud pendiente Alexandra.</t>
+          <t>Rails/policy en suite demo; Model Armor cloud pendiente P0-34. Cutover agentic: docs/handoffs/agentic-control-plane-cutover.md.</t>
         </is>
       </c>
     </row>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="I26" s="18" t="inlineStr">
         <is>
-          <t>JEV jerárquico en código; sin proveedor productivo nuevo; agentic no activado.</t>
+          <t>JEV jerárquico en código; sin proveedor productivo nuevo; agentic no activado en staging.</t>
         </is>
       </c>
     </row>
@@ -1846,7 +1846,7 @@
       </c>
       <c r="I27" s="18" t="inlineStr">
         <is>
-          <t>Policy/Tool Gateway evidenciado en tests demo; composición agentic no cerrada.</t>
+          <t>Policy/Tool Gateway + DisputePolicyEngine evidenciado (HITL REQUIRE_APPROVAL). Composición agentic staging no cerrada.</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="I28" s="18" t="inlineStr">
         <is>
-          <t>Structured RAG mantiene catálogo y adaptador BigQuery cerrados; no se habilita sin vistas y configuración aprobadas.</t>
+          <t>Structured RAG catálogo/adaptador BQ cerrados; KG_RAG_LOCAL_ENABLED=false en staging. No habilitar sin vistas/config aprobadas.</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="I30" s="18" t="inlineStr">
         <is>
-          <t>Output rail en suite demo/baseline; Model Armor cloud no verificado.</t>
+          <t>Output rail demo/baseline; Model Armor cloud no verificado (P0-34).</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="I34" s="18" t="inlineStr">
         <is>
-          <t>OTel/Langfuse Cloud US metadata-only, evaluadores baseline y persistencia BigQuery saneada implementados; Terraform declara dataset/tabla y preflight valida. Falta configurar secretos/flags autorizados, aplicar infraestructura y validar emisión en staging.</t>
+          <t>OTel/Langfuse/BQ eval implementados. Staging: correlador plano; OTEL/Langfuse off. Handoff: docs/handoffs/adr0020-ingest-and-tf.md + deploy/docs/live-telemetry-handoff.md.</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,11 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="I35" s="18" t="n"/>
+      <c r="I35" s="18" t="inlineStr">
+        <is>
+          <t>PENDING: API Model Armor habilitada; templates input/output no listados/verificados. Bloquea cutover agentic.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="36" customHeight="1" s="19">
       <c r="A36" s="26" t="inlineStr">
@@ -2308,7 +2312,7 @@
       </c>
       <c r="I37" s="26" t="inlineStr">
         <is>
-          <t>Terraform declara referencias Secret Manager versionables, IAM mínimo para backend (Firestore, BigQuery, Vertex y writer de evaluaciones) y VPC/Valkey; falta crear o importar recursos reales, revisar plan autorizado y aplicar.</t>
+          <t>TF declara SM/IAM/VPC/Valkey; falta import/create + plan/apply autorizado. Ver live-telemetry-handoff + handoff adr0020-ingest-and-tf.</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2359,7 @@
       </c>
       <c r="I38" s="26" t="inlineStr">
         <is>
-          <t>Cloud Run bankai-backend Ready (rev bankai-backend-00010-zxt, imagen sha256:76211ea7…0044) con chat baseline; Publish images 37366452866 success tras reintento por runner. Job bankai-pipeline creado sin ejecuciones observadas. DoD abierto: terraform plan/apply reconciliado (correlador→Secret Manager) y cadena de ingesta.</t>
+          <t>Cloud Run Ready (bankai-backend-00010-zxt); Job bankai-pipeline sin ejecuciones. DoD abierto: TF reconciliado + Job ejecutado + ingesta. Checklist docs/handoffs/adr0020-ingest-and-tf.md.</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2406,7 @@
       </c>
       <c r="I39" s="26" t="inlineStr">
         <is>
-          <t>ADR 0021</t>
+          <t>Bloqueado P0-16/P0-17/App Hosting. Interfaz smoke documentada en docs/handoffs/frontend-auth-smoke-p0-16-22-38.md.</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2451,11 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="I40" s="18" t="n"/>
+      <c r="I40" s="18" t="inlineStr">
+        <is>
+          <t>PENDING E2E integrado. Evidencia local HITL/casuísticas/policy + eval:gate en docs/handoffs/p0-39-e2e-checklist.md — no cierra DoD Playwright/k6/staging.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="83.25" customHeight="1" s="19">
       <c r="A41" s="26" t="inlineStr">
@@ -2539,7 +2547,7 @@
       </c>
       <c r="I42" s="26" t="inlineStr">
         <is>
-          <t>ADR 0020</t>
+          <t>ADR 0020: STS S3→GCS no desplegado. raw incompleto. Checklist docs/handoffs/adr0020-ingest-and-tf.md.</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2592,11 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="I43" s="18" t="n"/>
+      <c r="I43" s="18" t="inlineStr">
+        <is>
+          <t>Load GCS→raw BigQuery administrado abierto (ADR 0020).</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="36" customHeight="1" s="19">
       <c r="A44" s="26" t="inlineStr">
@@ -2627,7 +2639,11 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="I44" s="18" t="n"/>
+      <c r="I44" s="18" t="inlineStr">
+        <is>
+          <t>Hoja PENDING: stg/aux/cur ya materializados Fase 2 (prepare-20261005-canonical). Abierto: camino administrado raw→cur ADR 0020, no rehacer prepare canónico.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="36" customHeight="1" s="19">
       <c r="A45" s="26" t="inlineStr">
@@ -3423,7 +3439,7 @@
       </c>
       <c r="I62" s="26" t="inlineStr">
         <is>
-          <t>Ledger e idempotencia del contrato local están cubiertos; falta worker administrado ADR 0020 con Storage Transfer Service, Eventarc, Cloud Tasks, copia verified/ y carga BigQuery.</t>
+          <t>Idempotencia local OK; falta Eventarc→Tasks→worker→BQ. Ver handoff adr0020-ingest-and-tf.</t>
         </is>
       </c>
     </row>
@@ -3488,47 +3504,47 @@
       <c r="I68" s="32" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="18" t="inlineStr">
         <is>
           <t>P0-50</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="18" t="inlineStr">
         <is>
           <t>Comparar baseline vs control plane (A/B local).</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="18" t="inlineStr">
         <is>
           <t>CLI eval:compare con escenarios de prompts sintéticos (phase-1 Structured + phase-2 C1–C5/research). File sink local; sin persist BQ. Completitud técnica; juez semántico skipped.</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="18" t="inlineStr">
         <is>
           <t>Bun 1.4 · TypeScript · bun test · AgentControlService · BaselineConversationRunner</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E69" s="18" t="inlineStr">
         <is>
           <t>Ricardo</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="18" t="inlineStr">
         <is>
           <t>Done: bun run eval:compare genera runs/metrics/summary saneados en .local/eval-ab; same snapshot A/B; controlled gates vs baseline ungated; sin PII/prompts en artefactos; P0-48 intacto.</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G69" s="18" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H69" s="18" t="inlineStr">
         <is>
           <t>COMPLETED</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I69" s="18" t="inlineStr">
         <is>
           <t>Local A/B file sink listo (eval:compare). BQ vista segura/--persist diferido. P0-48 no reabierto.</t>
         </is>

</xml_diff>